<commit_message>
v1.3 of schematic with servo motor connection
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -5,13 +5,13 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEAE5BBC-4365-4AE5-B0CB-20AC8513012B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{EEAE5BBC-4365-4AE5-B0CB-20AC8513012B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A8F1AE6-9DDF-4311-A438-DD5C2984C6A5}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
   <si>
     <t>Link</t>
   </si>
@@ -235,6 +235,27 @@
   </si>
   <si>
     <t>Same Sky</t>
+  </si>
+  <si>
+    <t>TBP04R12-500-03BE</t>
+  </si>
+  <si>
+    <t>179-TBP04R12-50003BE</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/Same-Sky/TBP04R12-500-03BE?qs=TCDPyi3sCW0NaxY6tKwPhA%3D%3D</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/Infineon-Technologies/IRLML6402TRPBF?qs=9%252BKlkBgLFf0HuZuONx2Ewg%3D%3D</t>
+  </si>
+  <si>
+    <t>Infineon Technologies</t>
+  </si>
+  <si>
+    <t>IRLML6402TRPBF</t>
+  </si>
+  <si>
+    <t>942-IRLML6402TRPBF</t>
   </si>
 </sst>
 </file>
@@ -646,6 +667,45 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -659,45 +719,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1024,38 +1045,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="49"/>
+      <c r="B1" s="53"/>
       <c r="C1" s="19" t="s">
         <v>48</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="57" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="49"/>
+      <c r="B2" s="53"/>
       <c r="C2" s="20" t="s">
         <v>49</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="45" t="s">
+      <c r="H2" s="58" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
     </row>
     <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
@@ -1320,39 +1341,71 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>8</v>
       </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="36"/>
+      <c r="B12" s="28">
+        <v>1</v>
+      </c>
+      <c r="C12" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="H12" s="36">
+        <v>0.41299999999999998</v>
+      </c>
       <c r="I12" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J12" s="37"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.41299999999999998</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>9</v>
       </c>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="36"/>
+      <c r="B13" s="28">
+        <v>1</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="G13" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="H13" s="36">
+        <v>0.35299999999999998</v>
+      </c>
       <c r="I13" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J13" s="37"/>
+        <v>0.35299999999999998</v>
+      </c>
+      <c r="J13" s="37" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
@@ -1457,13 +1510,13 @@
       <c r="J19" s="39"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G20" s="46" t="s">
+      <c r="G20" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="H20" s="46"/>
+      <c r="H20" s="59"/>
       <c r="I20" s="12">
         <f>SUM(I5:I19)</f>
-        <v>13.641999999999999</v>
+        <v>14.407999999999999</v>
       </c>
       <c r="J20" s="4"/>
     </row>
@@ -1475,101 +1528,101 @@
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="15"/>
-      <c r="G21" s="47" t="s">
+      <c r="G21" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="H21" s="47"/>
+      <c r="H21" s="60"/>
       <c r="I21" s="10">
         <f>I20*0.19</f>
-        <v>2.59198</v>
+        <v>2.73752</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="50" t="s">
+      <c r="A22" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="51"/>
+      <c r="B22" s="55"/>
       <c r="C22" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="51" t="s">
+      <c r="D22" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="54"/>
-      <c r="G22" s="47" t="s">
+      <c r="E22" s="56"/>
+      <c r="G22" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="H22" s="47"/>
+      <c r="H22" s="60"/>
       <c r="I22" s="11">
         <f>I20*1.19</f>
-        <v>16.233979999999999</v>
+        <v>17.145519999999998</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="52" t="s">
+      <c r="A23" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="53"/>
+      <c r="B23" s="45"/>
       <c r="C23" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="57" t="s">
+      <c r="D23" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="58"/>
+      <c r="E23" s="49"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="52" t="s">
+      <c r="A24" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="53"/>
+      <c r="B24" s="45"/>
       <c r="C24" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="57" t="s">
+      <c r="D24" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="58"/>
+      <c r="E24" s="49"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="52" t="s">
+      <c r="A25" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="53"/>
+      <c r="B25" s="45"/>
       <c r="C25" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="57" t="s">
+      <c r="D25" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="58"/>
+      <c r="E25" s="49"/>
       <c r="H25" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="55" t="s">
+      <c r="A26" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="56"/>
+      <c r="B26" s="47"/>
       <c r="C26" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="59" t="s">
+      <c r="D26" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="60"/>
+      <c r="E26" s="51"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="55" t="s">
+      <c r="A27" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="56"/>
+      <c r="B27" s="47"/>
       <c r="C27" s="18"/>
-      <c r="D27" s="59" t="s">
+      <c r="D27" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="E27" s="60"/>
+      <c r="E27" s="51"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
@@ -1669,6 +1722,16 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="D22:E22"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A27:B27"/>
@@ -1678,16 +1741,6 @@
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F19" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -1703,9 +1756,11 @@
     <hyperlink ref="J7" r:id="rId6" xr:uid="{4987D0AF-D5AF-4E59-98D4-4D42395D39EC}"/>
     <hyperlink ref="J6" r:id="rId7" xr:uid="{9F9E23C2-0CE5-4F54-A453-2FB0482436B8}"/>
     <hyperlink ref="J5" r:id="rId8" xr:uid="{98A04EE6-D62B-4687-AC62-05CBC3BC7F14}"/>
+    <hyperlink ref="J11" r:id="rId9" xr:uid="{E0F5E5CE-E58B-4232-8792-169F1500BA12}"/>
+    <hyperlink ref="J13" r:id="rId10" xr:uid="{85611FA3-DA6B-4401-BC4A-CB8B8F5F9061}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId9"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId11"/>
   <headerFooter>
     <oddHeader>&amp;CParts list
 Practical Electronics</oddHeader>

</xml_diff>

<commit_message>
added NPN to BOM
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Projects\pe04\schematic-design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{EEAE5BBC-4365-4AE5-B0CB-20AC8513012B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A8F1AE6-9DDF-4311-A438-DD5C2984C6A5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161CBEA3-A91F-4564-AED2-E40A4C628EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="79">
   <si>
     <t>Link</t>
   </si>
@@ -256,6 +256,21 @@
   </si>
   <si>
     <t>942-IRLML6402TRPBF</t>
+  </si>
+  <si>
+    <t>CDIL</t>
+  </si>
+  <si>
+    <t>Bipolartransistor</t>
+  </si>
+  <si>
+    <t>BC547B</t>
+  </si>
+  <si>
+    <t>BC 547B</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.de/de/de/shop/produkt/bipolartransistor_npn_45v_0_1a_0_5w_to-92-5006</t>
   </si>
 </sst>
 </file>
@@ -667,12 +682,41 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -690,35 +734,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1027,58 +1042,58 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J49"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="7.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="8" width="8.7109375" customWidth="1"/>
-    <col min="9" max="9" width="6.5703125" customWidth="1"/>
-    <col min="10" max="10" width="55.28515625" customWidth="1"/>
-    <col min="13" max="13" width="12.28515625" customWidth="1"/>
-    <col min="20" max="20" width="9.42578125" customWidth="1"/>
-    <col min="21" max="21" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" customWidth="1"/>
+    <col min="9" max="9" width="6.5546875" customWidth="1"/>
+    <col min="10" max="10" width="55.33203125" customWidth="1"/>
+    <col min="13" max="13" width="12.33203125" customWidth="1"/>
+    <col min="20" max="20" width="9.44140625" customWidth="1"/>
+    <col min="21" max="21" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="53"/>
+      <c r="B1" s="49"/>
       <c r="C1" s="19" t="s">
         <v>48</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="57" t="s">
+      <c r="H1" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="53"/>
+      <c r="B2" s="49"/>
       <c r="C2" s="20" t="s">
         <v>49</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="58" t="s">
+      <c r="H2" s="45" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-    </row>
-    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+    </row>
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -1110,7 +1125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="42">
         <v>1</v>
       </c>
@@ -1143,7 +1158,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="43">
         <v>2</v>
       </c>
@@ -1176,7 +1191,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="43">
         <v>3</v>
       </c>
@@ -1209,7 +1224,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="7">
         <v>4</v>
       </c>
@@ -1242,7 +1257,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="7">
         <v>5</v>
       </c>
@@ -1275,7 +1290,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="7">
         <v>6</v>
       </c>
@@ -1308,7 +1323,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>7</v>
       </c>
@@ -1341,7 +1356,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>8</v>
       </c>
@@ -1374,7 +1389,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>9</v>
       </c>
@@ -1407,24 +1422,40 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>10</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="36"/>
+      <c r="B14" s="28">
+        <v>1</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="H14" s="36">
+        <v>0.04</v>
+      </c>
       <c r="I14" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J14" s="37"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+        <v>0.04</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>11</v>
       </c>
@@ -1441,7 +1472,7 @@
       </c>
       <c r="J15" s="37"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>12</v>
       </c>
@@ -1458,7 +1489,7 @@
       </c>
       <c r="J16" s="37"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>13</v>
       </c>
@@ -1475,7 +1506,7 @@
       </c>
       <c r="J17" s="37"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>14</v>
       </c>
@@ -1492,7 +1523,7 @@
       </c>
       <c r="J18" s="37"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>15</v>
       </c>
@@ -1509,18 +1540,18 @@
       </c>
       <c r="J19" s="39"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G20" s="59" t="s">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G20" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="H20" s="59"/>
+      <c r="H20" s="46"/>
       <c r="I20" s="12">
         <f>SUM(I5:I19)</f>
-        <v>14.407999999999999</v>
+        <v>14.447999999999999</v>
       </c>
       <c r="J20" s="4"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
         <v>24</v>
       </c>
@@ -1528,103 +1559,103 @@
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="15"/>
-      <c r="G21" s="60" t="s">
+      <c r="G21" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="H21" s="60"/>
+      <c r="H21" s="47"/>
       <c r="I21" s="10">
         <f>I20*0.19</f>
-        <v>2.73752</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="54" t="s">
+        <v>2.7451199999999996</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="55"/>
+      <c r="B22" s="51"/>
       <c r="C22" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="55" t="s">
+      <c r="D22" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="56"/>
-      <c r="G22" s="60" t="s">
+      <c r="E22" s="54"/>
+      <c r="G22" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="H22" s="60"/>
+      <c r="H22" s="47"/>
       <c r="I22" s="11">
         <f>I20*1.19</f>
-        <v>17.145519999999998</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="44" t="s">
+        <v>17.193119999999997</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="45"/>
+      <c r="B23" s="53"/>
       <c r="C23" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="49"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="44" t="s">
+      <c r="E23" s="58"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="45"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="48" t="s">
+      <c r="D24" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="49"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="44" t="s">
+      <c r="E24" s="58"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="45"/>
+      <c r="B25" s="53"/>
       <c r="C25" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="48" t="s">
+      <c r="D25" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="49"/>
+      <c r="E25" s="58"/>
       <c r="H25" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="46" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="47"/>
+      <c r="B26" s="56"/>
       <c r="C26" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="50" t="s">
+      <c r="D26" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="51"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="46" t="s">
+      <c r="E26" s="60"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="47"/>
+      <c r="B27" s="56"/>
       <c r="C27" s="18"/>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="E27" s="51"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E27" s="60"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="1"/>
@@ -1636,7 +1667,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="2"/>
@@ -1648,7 +1679,7 @@
       <c r="I43" s="1"/>
       <c r="J43" s="3"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="2"/>
@@ -1660,7 +1691,7 @@
       <c r="I44" s="1"/>
       <c r="J44" s="3"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="2"/>
@@ -1672,7 +1703,7 @@
       <c r="I45" s="1"/>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="2"/>
@@ -1684,7 +1715,7 @@
       <c r="I46" s="1"/>
       <c r="J46" s="3"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1696,7 +1727,7 @@
       <c r="I47" s="1"/>
       <c r="J47" s="3"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="2"/>
@@ -1708,7 +1739,7 @@
       <c r="I48" s="1"/>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="2"/>
@@ -1722,16 +1753,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="D22:E22"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A27:B27"/>
@@ -1741,8 +1762,18 @@
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="D26:E26"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F19" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$A$23:$A$27</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Updated diode for safety margin, added diodes and servo to Partslist_Group_PE04_2.xlsx
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Projects\pe04\schematic-design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161CBEA3-A91F-4564-AED2-E40A4C628EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{161CBEA3-A91F-4564-AED2-E40A4C628EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54EA14C4-37E7-4905-A824-B3ED336D4F05}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="93">
   <si>
     <t>Link</t>
   </si>
@@ -271,6 +271,48 @@
   </si>
   <si>
     <t>https://www.reichelt.de/de/de/shop/produkt/bipolartransistor_npn_45v_0_1a_0_5w_to-92-5006</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.com/de/en/shop/product/schottky_diode_do201ad_40_v_3_a-41852</t>
+  </si>
+  <si>
+    <t>1N5822</t>
+  </si>
+  <si>
+    <t>Schottky diode, DO201AD, 40 V, 3 A</t>
+  </si>
+  <si>
+    <t>1N 5822</t>
+  </si>
+  <si>
+    <t>MIC</t>
+  </si>
+  <si>
+    <t>Schottky diode, DO41, 40 V, 1 A</t>
+  </si>
+  <si>
+    <t>1N5819</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.com/de/en/shop/product/schottky_diode_do41_40_v_1_a-41850</t>
+  </si>
+  <si>
+    <t>1N 5819</t>
+  </si>
+  <si>
+    <t>LUNSURE</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/DFRobot/SER0050?qs=zW32dvEIR3t5syqsDiJx%2Fw%3D%3D</t>
+  </si>
+  <si>
+    <t>SER0050</t>
+  </si>
+  <si>
+    <t>426-SER0050</t>
+  </si>
+  <si>
+    <t>DFRobot</t>
   </si>
 </sst>
 </file>
@@ -682,6 +724,45 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -695,45 +776,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1042,58 +1084,58 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J49"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="4.88671875" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="7.6640625" customWidth="1"/>
-    <col min="7" max="7" width="12.88671875" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" customWidth="1"/>
-    <col min="10" max="10" width="55.33203125" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" customWidth="1"/>
-    <col min="20" max="20" width="9.44140625" customWidth="1"/>
-    <col min="21" max="21" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="4.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" customWidth="1"/>
+    <col min="9" max="9" width="6.5703125" customWidth="1"/>
+    <col min="10" max="10" width="55.28515625" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" customWidth="1"/>
+    <col min="20" max="20" width="9.42578125" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="49"/>
+      <c r="B1" s="53"/>
       <c r="C1" s="19" t="s">
         <v>48</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="57" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="49"/>
+      <c r="B2" s="53"/>
       <c r="C2" s="20" t="s">
         <v>49</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="45" t="s">
+      <c r="H2" s="58" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+    </row>
+    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
@@ -1125,7 +1167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="42">
         <v>1</v>
       </c>
@@ -1158,7 +1200,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="43">
         <v>2</v>
       </c>
@@ -1191,7 +1233,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="43">
         <v>3</v>
       </c>
@@ -1224,7 +1266,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>4</v>
       </c>
@@ -1257,7 +1299,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>5</v>
       </c>
@@ -1290,7 +1332,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>6</v>
       </c>
@@ -1323,7 +1365,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>7</v>
       </c>
@@ -1356,7 +1398,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>8</v>
       </c>
@@ -1389,7 +1431,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>9</v>
       </c>
@@ -1422,7 +1464,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>10</v>
       </c>
@@ -1455,58 +1497,106 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <v>11</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="36"/>
+      <c r="B15" s="28">
+        <v>2</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="H15" s="36">
+        <v>0.15</v>
+      </c>
       <c r="I15" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J15" s="37"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>0.3</v>
+      </c>
+      <c r="J15" s="37" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>12</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="36"/>
+      <c r="B16" s="28">
+        <v>1</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>87</v>
+      </c>
+      <c r="H16" s="36">
+        <v>0.05</v>
+      </c>
       <c r="I16" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J16" s="37"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+        <v>0.05</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>13</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="36"/>
+      <c r="B17" s="28">
+        <v>1</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="G17" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="H17" s="36">
+        <v>5.16</v>
+      </c>
       <c r="I17" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J17" s="37"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+        <v>5.16</v>
+      </c>
+      <c r="J17" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>14</v>
       </c>
@@ -1523,7 +1613,7 @@
       </c>
       <c r="J18" s="37"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>15</v>
       </c>
@@ -1540,18 +1630,18 @@
       </c>
       <c r="J19" s="39"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G20" s="46" t="s">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G20" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="H20" s="46"/>
+      <c r="H20" s="59"/>
       <c r="I20" s="12">
         <f>SUM(I5:I19)</f>
-        <v>14.447999999999999</v>
+        <v>19.957999999999998</v>
       </c>
       <c r="J20" s="4"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>24</v>
       </c>
@@ -1559,103 +1649,103 @@
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="15"/>
-      <c r="G21" s="47" t="s">
+      <c r="G21" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="H21" s="47"/>
+      <c r="H21" s="60"/>
       <c r="I21" s="10">
         <f>I20*0.19</f>
-        <v>2.7451199999999996</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="50" t="s">
+        <v>3.7920199999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="51"/>
+      <c r="B22" s="55"/>
       <c r="C22" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="51" t="s">
+      <c r="D22" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="54"/>
-      <c r="G22" s="47" t="s">
+      <c r="E22" s="56"/>
+      <c r="G22" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="H22" s="47"/>
+      <c r="H22" s="60"/>
       <c r="I22" s="11">
         <f>I20*1.19</f>
-        <v>17.193119999999997</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="52" t="s">
+        <v>23.750019999999996</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="53"/>
+      <c r="B23" s="45"/>
       <c r="C23" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="57" t="s">
+      <c r="D23" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="58"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="52" t="s">
+      <c r="E23" s="49"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="53"/>
+      <c r="B24" s="45"/>
       <c r="C24" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="57" t="s">
+      <c r="D24" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="58"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="52" t="s">
+      <c r="E24" s="49"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="53"/>
+      <c r="B25" s="45"/>
       <c r="C25" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="57" t="s">
+      <c r="D25" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="58"/>
+      <c r="E25" s="49"/>
       <c r="H25" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="55" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="56"/>
+      <c r="B26" s="47"/>
       <c r="C26" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="59" t="s">
+      <c r="D26" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="60"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="55" t="s">
+      <c r="E26" s="51"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="56"/>
+      <c r="B27" s="47"/>
       <c r="C27" s="18"/>
-      <c r="D27" s="59" t="s">
+      <c r="D27" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="E27" s="60"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E27" s="51"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="1"/>
@@ -1667,7 +1757,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="2"/>
@@ -1679,7 +1769,7 @@
       <c r="I43" s="1"/>
       <c r="J43" s="3"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="2"/>
@@ -1691,7 +1781,7 @@
       <c r="I44" s="1"/>
       <c r="J44" s="3"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="2"/>
@@ -1703,7 +1793,7 @@
       <c r="I45" s="1"/>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="2"/>
@@ -1715,7 +1805,7 @@
       <c r="I46" s="1"/>
       <c r="J46" s="3"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1727,7 +1817,7 @@
       <c r="I47" s="1"/>
       <c r="J47" s="3"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="2"/>
@@ -1739,7 +1829,7 @@
       <c r="I48" s="1"/>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="2"/>
@@ -1753,6 +1843,16 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="D22:E22"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A27:B27"/>
@@ -1762,18 +1862,8 @@
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F19" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$A$23:$A$27</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Shifting to USB port, so added port and UART, but UART not connected
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{161CBEA3-A91F-4564-AED2-E40A4C628EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54EA14C4-37E7-4905-A824-B3ED336D4F05}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{161CBEA3-A91F-4564-AED2-E40A4C628EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BD6E43D-ADA7-44A9-AE5E-503BD3A152D4}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="97">
   <si>
     <t>Link</t>
   </si>
@@ -225,15 +225,6 @@
     <t>onsemi</t>
   </si>
   <si>
-    <t>https://www.mouser.de/ProductDetail/Same-Sky/UJ20-C-H-G-TH-P16-TR?qs=IKkN%2F947nfDgv1IMBq%252Bdzg%3D%3D</t>
-  </si>
-  <si>
-    <t>179-UJ20CHGTHP16TR</t>
-  </si>
-  <si>
-    <t>UJ20-C-H-G-TH-P16-TR</t>
-  </si>
-  <si>
     <t>Same Sky</t>
   </si>
   <si>
@@ -313,6 +304,27 @@
   </si>
   <si>
     <t>DFRobot</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/Same-Sky/UJ2-B-HR-G-TH?qs=HoCaDK9Nz5cuzuu5C%2FN7nw%3D%3D</t>
+  </si>
+  <si>
+    <t>179-UJ2-B-HR-G-TH</t>
+  </si>
+  <si>
+    <t>UJ2-B-HR-G-TH</t>
+  </si>
+  <si>
+    <t>895-FT230XS-U</t>
+  </si>
+  <si>
+    <t>FT230XS-U</t>
+  </si>
+  <si>
+    <t>FTDI</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/FTDI/FT230XS-U?qs=sGAEpiMZZMsX%252BY3VKDPZyP5eriYtgtkavaou6tk%2F0oE%3D</t>
   </si>
 </sst>
 </file>
@@ -724,12 +736,41 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -747,35 +788,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -794,6 +806,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1102,38 +1118,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="53"/>
+      <c r="B1" s="49"/>
       <c r="C1" s="19" t="s">
         <v>48</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="57" t="s">
+      <c r="H1" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="53"/>
+      <c r="B2" s="49"/>
       <c r="C2" s="20" t="s">
         <v>49</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="58" t="s">
+      <c r="H2" s="45" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
     </row>
     <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
@@ -1365,7 +1381,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>7</v>
       </c>
@@ -1373,29 +1389,29 @@
         <v>1</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="F11" s="28" t="s">
         <v>30</v>
       </c>
       <c r="G11" s="28" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="H11" s="36">
-        <v>0.80800000000000005</v>
+        <v>1.29</v>
       </c>
       <c r="I11" s="35">
         <f>B11*H11</f>
-        <v>0.80800000000000005</v>
+        <v>1.29</v>
       </c>
       <c r="J11" s="37" t="s">
-        <v>63</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -1406,19 +1422,19 @@
         <v>1</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E12" s="28" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F12" s="28" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="28" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H12" s="36">
         <v>0.41299999999999998</v>
@@ -1428,7 +1444,7 @@
         <v>0.41299999999999998</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -1439,19 +1455,19 @@
         <v>1</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E13" s="28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F13" s="28" t="s">
         <v>30</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H13" s="36">
         <v>0.35299999999999998</v>
@@ -1461,7 +1477,7 @@
         <v>0.35299999999999998</v>
       </c>
       <c r="J13" s="37" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -1472,19 +1488,19 @@
         <v>1</v>
       </c>
       <c r="C14" s="28" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E14" s="28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F14" s="28" t="s">
         <v>29</v>
       </c>
       <c r="G14" s="28" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H14" s="36">
         <v>0.04</v>
@@ -1494,7 +1510,7 @@
         <v>0.04</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="60" x14ac:dyDescent="0.25">
@@ -1505,19 +1521,19 @@
         <v>2</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E15" s="28" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F15" s="28" t="s">
         <v>31</v>
       </c>
       <c r="G15" s="28" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H15" s="36">
         <v>0.15</v>
@@ -1527,7 +1543,7 @@
         <v>0.3</v>
       </c>
       <c r="J15" s="37" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -1538,19 +1554,19 @@
         <v>1</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E16" s="28" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F16" s="28" t="s">
         <v>31</v>
       </c>
       <c r="G16" s="28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H16" s="36">
         <v>0.05</v>
@@ -1560,7 +1576,7 @@
         <v>0.05</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -1571,19 +1587,19 @@
         <v>1</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F17" s="28" t="s">
         <v>30</v>
       </c>
       <c r="G17" s="28" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H17" s="36">
         <v>5.16</v>
@@ -1593,25 +1609,41 @@
         <v>5.16</v>
       </c>
       <c r="J17" s="37" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>14</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="36"/>
+      <c r="B18" s="28">
+        <v>1</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="E18" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18" s="36">
+        <v>1.7</v>
+      </c>
       <c r="I18" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J18" s="37"/>
+        <v>1.7</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
@@ -1631,13 +1663,13 @@
       <c r="J19" s="39"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G20" s="59" t="s">
+      <c r="G20" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="H20" s="59"/>
+      <c r="H20" s="46"/>
       <c r="I20" s="12">
         <f>SUM(I5:I19)</f>
-        <v>19.957999999999998</v>
+        <v>22.139999999999997</v>
       </c>
       <c r="J20" s="4"/>
     </row>
@@ -1649,101 +1681,101 @@
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="15"/>
-      <c r="G21" s="60" t="s">
+      <c r="G21" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="H21" s="60"/>
+      <c r="H21" s="47"/>
       <c r="I21" s="10">
         <f>I20*0.19</f>
-        <v>3.7920199999999999</v>
+        <v>4.2065999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="55"/>
+      <c r="B22" s="51"/>
       <c r="C22" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="55" t="s">
+      <c r="D22" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="E22" s="56"/>
-      <c r="G22" s="60" t="s">
+      <c r="E22" s="54"/>
+      <c r="G22" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="H22" s="60"/>
+      <c r="H22" s="47"/>
       <c r="I22" s="11">
         <f>I20*1.19</f>
-        <v>23.750019999999996</v>
+        <v>26.346599999999995</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="44" t="s">
+      <c r="A23" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="45"/>
+      <c r="B23" s="53"/>
       <c r="C23" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="49"/>
+      <c r="E23" s="58"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="45"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="48" t="s">
+      <c r="D24" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="49"/>
+      <c r="E24" s="58"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="44" t="s">
+      <c r="A25" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="45"/>
+      <c r="B25" s="53"/>
       <c r="C25" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="48" t="s">
+      <c r="D25" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="49"/>
+      <c r="E25" s="58"/>
       <c r="H25" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="47"/>
+      <c r="B26" s="56"/>
       <c r="C26" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="50" t="s">
+      <c r="D26" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="E26" s="51"/>
+      <c r="E26" s="60"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="47"/>
+      <c r="B27" s="56"/>
       <c r="C27" s="18"/>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="E27" s="51"/>
+      <c r="E27" s="60"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
@@ -1843,16 +1875,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="D22:E22"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A27:B27"/>
@@ -1862,6 +1884,16 @@
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="D26:E26"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5:F19" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>

<commit_message>
Made first draft of pcb design, modified existing library symbol, changes to BOM, changes to schematic
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{23A68183-9883-4898-B30F-B2C1DE7AC4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{610BD965-C685-40A0-9899-7A03DAA8771C}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="13_ncr:1_{23A68183-9883-4898-B30F-B2C1DE7AC4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF5B5E48-CE05-4F58-8273-2AF4472BC6F5}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="80">
   <si>
     <t>Link</t>
   </si>
@@ -141,18 +141,12 @@
     <t>04</t>
   </si>
   <si>
-    <t>23/10/2025</t>
-  </si>
-  <si>
     <t>Justin Chin Cheong, Abhinav Kothari</t>
   </si>
   <si>
     <t>Knock Lock</t>
   </si>
   <si>
-    <t>Keystone Electronics</t>
-  </si>
-  <si>
     <t>https://www.mouser.de/ProductDetail/Microchip-Technology/LM2575-3.3WT?qs=kh6iOki%2FeLFAZSEMjMNbiQ%3D%3D</t>
   </si>
   <si>
@@ -165,15 +159,6 @@
     <t>Microchip Technology</t>
   </si>
   <si>
-    <t>534-2477</t>
-  </si>
-  <si>
-    <t>https://www.mouser.de/ProductDetail/Keystone-Electronics/2477?qs=Q3RoVmURDolEbXnNenQutg%3D%3D</t>
-  </si>
-  <si>
-    <t>Same Sky</t>
-  </si>
-  <si>
     <t>https://www.mouser.de/ProductDetail/Infineon-Technologies/IRLML6402TRPBF?qs=9%252BKlkBgLFf0HuZuONx2Ewg%3D%3D</t>
   </si>
   <si>
@@ -213,18 +198,6 @@
     <t>DFRobot</t>
   </si>
   <si>
-    <t>https://www.mouser.de/ProductDetail/Same-Sky/UJ2-B-HR-G-TH?qs=HoCaDK9Nz5cuzuu5C%2FN7nw%3D%3D</t>
-  </si>
-  <si>
-    <t>179-UJ2-B-HR-G-TH</t>
-  </si>
-  <si>
-    <t>UJ2-B-HR-G-TH</t>
-  </si>
-  <si>
-    <t>2477 Battery Holder</t>
-  </si>
-  <si>
     <t>LM2575-3.3WT Voltage Regulator</t>
   </si>
   <si>
@@ -234,9 +207,6 @@
     <t>SER0050 Servo Motor</t>
   </si>
   <si>
-    <t>UJ2-B-HR-G-TH USB B Port</t>
-  </si>
-  <si>
     <t>https://eu.mouser.com/ProductDetail/Vishay-BC-Components/K104K15X7RF5WH5?qs=sGAEpiMZZMuMW9TJLBQkXstS33ZYjGCMau7NPGXn%2F5U%3D</t>
   </si>
   <si>
@@ -280,6 +250,30 @@
   </si>
   <si>
     <t>https://www.mouser.de/ProductDetail/Coilcraft/RFC0810B-334KE?qs=ZYnrCdKdyedaHxMGgKKlpw%3D%3D</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/GCT/USB3145-30-1-A?qs=KUoIvG%2F9IlYD1lvSRu5iyg%3D%3D</t>
+  </si>
+  <si>
+    <t>640-USB3145-30-1-A</t>
+  </si>
+  <si>
+    <t>USB3145-30-1-A</t>
+  </si>
+  <si>
+    <t>GCT</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/Eagle-Plastic-Devices/12BH342A-GR?qs=GYzcNiWpw3fGsZG%2F3838jw%3D%3D</t>
+  </si>
+  <si>
+    <t>12BH342A-GR</t>
+  </si>
+  <si>
+    <t>12BH342A-GR Battery Holder</t>
+  </si>
+  <si>
+    <t>Eagle Plastic Devices</t>
   </si>
 </sst>
 </file>
@@ -655,9 +649,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -668,59 +659,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -739,6 +677,60 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1049,58 +1041,58 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J54"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="4.88671875" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="7.6640625" customWidth="1"/>
-    <col min="7" max="7" width="12.88671875" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" customWidth="1"/>
-    <col min="10" max="10" width="55.33203125" customWidth="1"/>
-    <col min="13" max="13" width="12.33203125" customWidth="1"/>
-    <col min="20" max="20" width="9.44140625" customWidth="1"/>
-    <col min="21" max="21" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="4.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" customWidth="1"/>
+    <col min="9" max="9" width="6.5703125" customWidth="1"/>
+    <col min="10" max="10" width="55.28515625" customWidth="1"/>
+    <col min="13" max="13" width="12.28515625" customWidth="1"/>
+    <col min="20" max="20" width="9.42578125" customWidth="1"/>
+    <col min="21" max="21" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="39"/>
+      <c r="B1" s="43"/>
       <c r="C1" s="16" t="s">
         <v>34</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="H1" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="17" t="s">
-        <v>35</v>
+      <c r="B2" s="43"/>
+      <c r="C2" s="17">
+        <v>45788</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H2" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+    </row>
+    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -1132,40 +1124,40 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
         <v>1</v>
       </c>
       <c r="B5" s="18">
         <v>1</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>38</v>
+      <c r="C5" s="55" t="s">
+        <v>79</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" s="21">
-        <v>2477</v>
+        <v>78</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>77</v>
       </c>
       <c r="F5" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="30" t="s">
-        <v>43</v>
+      <c r="G5" s="29" t="s">
+        <v>77</v>
       </c>
       <c r="H5" s="23">
-        <v>1.87</v>
+        <v>1.54</v>
       </c>
       <c r="I5" s="24">
-        <f>B5*H5</f>
-        <v>1.87</v>
+        <f t="shared" ref="I5:I11" si="0">B5*H5</f>
+        <v>1.54</v>
       </c>
       <c r="J5" s="22" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
         <v>2</v>
       </c>
@@ -1173,32 +1165,32 @@
         <v>1</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F6" s="18" t="s">
         <v>30</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H6" s="23">
         <v>1.48</v>
       </c>
       <c r="I6" s="24">
-        <f>B6*H6</f>
+        <f t="shared" si="0"/>
         <v>1.48</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6">
         <v>3</v>
       </c>
@@ -1206,32 +1198,32 @@
         <v>1</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="H7" s="25">
-        <v>1.29</v>
+        <v>0.66200000000000003</v>
       </c>
       <c r="I7" s="24">
-        <f>B7*H7</f>
-        <v>1.29</v>
+        <f t="shared" si="0"/>
+        <v>0.66200000000000003</v>
       </c>
       <c r="J7" s="26" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>4</v>
       </c>
@@ -1239,32 +1231,32 @@
         <v>1</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H8" s="25">
         <v>0.35299999999999998</v>
       </c>
       <c r="I8" s="24">
-        <f>B8*H8</f>
+        <f t="shared" si="0"/>
         <v>0.35299999999999998</v>
       </c>
       <c r="J8" s="26" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>5</v>
       </c>
@@ -1272,32 +1264,32 @@
         <v>4</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>31</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="H9" s="25">
         <v>0.15</v>
       </c>
       <c r="I9" s="24">
-        <f>B9*H9</f>
+        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
         <v>6</v>
       </c>
@@ -1305,32 +1297,32 @@
         <v>1</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F10" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H10" s="25">
         <v>5.16</v>
       </c>
       <c r="I10" s="24">
-        <f>B10*H10</f>
+        <f t="shared" si="0"/>
         <v>5.16</v>
       </c>
       <c r="J10" s="26" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="6">
         <v>7</v>
       </c>
@@ -1338,249 +1330,249 @@
         <v>4</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="F11" s="20" t="s">
         <v>30</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H11" s="27">
         <v>0.13</v>
       </c>
       <c r="I11" s="24">
-        <f>B11*H11</f>
+        <f t="shared" si="0"/>
         <v>0.52</v>
       </c>
       <c r="J11" s="28" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>8</v>
       </c>
-      <c r="B12" s="31">
+      <c r="B12" s="30">
         <v>1</v>
       </c>
-      <c r="C12" s="31" t="s">
-        <v>76</v>
+      <c r="C12" s="30" t="s">
+        <v>66</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="H12" s="25">
         <v>0.16</v>
       </c>
       <c r="I12" s="24">
-        <f t="shared" ref="I12:I13" si="0">B12*H12</f>
+        <f t="shared" ref="I12:I13" si="1">B12*H12</f>
         <v>0.16</v>
       </c>
       <c r="J12" s="26" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>9</v>
       </c>
       <c r="B13" s="19">
         <v>1</v>
       </c>
-      <c r="C13" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="D13" s="31" t="s">
-        <v>77</v>
+      <c r="C13" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>67</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H13" s="25">
         <v>1.26</v>
       </c>
-      <c r="I13" s="51">
-        <f t="shared" si="0"/>
+      <c r="I13" s="33">
+        <f t="shared" si="1"/>
         <v>1.26</v>
       </c>
       <c r="J13" s="26" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>10</v>
       </c>
-      <c r="B14" s="52"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="52"/>
-      <c r="H14" s="52"/>
-      <c r="I14" s="52"/>
-      <c r="J14" s="52"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>11</v>
       </c>
-      <c r="B15" s="52"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="52"/>
-      <c r="I15" s="52"/>
-      <c r="J15" s="52"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="34"/>
+      <c r="J15" s="34"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
         <v>12</v>
       </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="52"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="52"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
+      <c r="J16" s="34"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="6">
         <v>13</v>
       </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="52"/>
-      <c r="G17" s="52"/>
-      <c r="H17" s="52"/>
-      <c r="I17" s="52"/>
-      <c r="J17" s="52"/>
-    </row>
-    <row r="18" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
+      <c r="J17" s="34"/>
+    </row>
+    <row r="18" spans="1:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>14</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="52"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="52"/>
-      <c r="G18" s="52"/>
-      <c r="H18" s="52"/>
-      <c r="I18" s="52"/>
-      <c r="J18" s="52"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34"/>
+      <c r="J18" s="34"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="6">
         <v>15</v>
       </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52"/>
-      <c r="E19" s="52"/>
-      <c r="F19" s="52"/>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52"/>
-      <c r="I19" s="52"/>
-      <c r="J19" s="52"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
+      <c r="J19" s="34"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>16</v>
       </c>
-      <c r="B20" s="52"/>
-      <c r="C20" s="52"/>
-      <c r="D20" s="52"/>
-      <c r="E20" s="52"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="52"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="52"/>
-      <c r="J20" s="52"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="34"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
         <v>17</v>
       </c>
-      <c r="B21" s="52"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="52"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="52"/>
-      <c r="J21" s="52"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
+      <c r="J21" s="34"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="6">
         <v>18</v>
       </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="52"/>
-      <c r="I22" s="52"/>
-      <c r="J22" s="52"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="34"/>
+      <c r="J22" s="34"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>19</v>
       </c>
-      <c r="B23" s="53"/>
-      <c r="C23" s="53"/>
-      <c r="D23" s="53"/>
-      <c r="E23" s="53"/>
-      <c r="F23" s="53"/>
-      <c r="G23" s="53"/>
-      <c r="H23" s="54"/>
-      <c r="I23" s="54"/>
-      <c r="J23" s="55"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G25" s="36" t="s">
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="35"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="37"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G25" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="H25" s="36"/>
+      <c r="H25" s="40"/>
       <c r="I25" s="9">
         <f>SUM(I5:I23)</f>
-        <v>12.693</v>
-      </c>
-      <c r="J25" s="33"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+        <v>11.734999999999999</v>
+      </c>
+      <c r="J25" s="32"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>24</v>
       </c>
@@ -1588,106 +1580,106 @@
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
       <c r="E26" s="12"/>
-      <c r="G26" s="37" t="s">
+      <c r="G26" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="H26" s="37"/>
+      <c r="H26" s="41"/>
       <c r="I26" s="7">
         <f>I25*0.19</f>
-        <v>2.41167</v>
-      </c>
-      <c r="J26" s="33"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="40" t="s">
+        <v>2.2296499999999999</v>
+      </c>
+      <c r="J26" s="32"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="41"/>
+      <c r="B27" s="45"/>
       <c r="C27" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="44"/>
-      <c r="G27" s="37" t="s">
+      <c r="E27" s="48"/>
+      <c r="G27" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="H27" s="37"/>
+      <c r="H27" s="41"/>
       <c r="I27" s="8">
         <f>I25*1.19</f>
-        <v>15.104669999999999</v>
-      </c>
-      <c r="J27" s="33"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="42" t="s">
+        <v>13.964649999999999</v>
+      </c>
+      <c r="J27" s="32"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="43"/>
+      <c r="B28" s="47"/>
       <c r="C28" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="47" t="s">
+      <c r="D28" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="E28" s="48"/>
-      <c r="I28" s="32"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" s="42" t="s">
+      <c r="E28" s="52"/>
+      <c r="I28" s="31"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="43"/>
+      <c r="B29" s="47"/>
       <c r="C29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="47" t="s">
+      <c r="D29" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="48"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="42" t="s">
+      <c r="E29" s="52"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="43"/>
+      <c r="B30" s="47"/>
       <c r="C30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="47" t="s">
+      <c r="D30" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="E30" s="48"/>
+      <c r="E30" s="52"/>
       <c r="H30" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="45" t="s">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="46"/>
+      <c r="B31" s="50"/>
       <c r="C31" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="49" t="s">
+      <c r="D31" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="E31" s="50"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" s="45" t="s">
+      <c r="E31" s="54"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="46"/>
+      <c r="B32" s="50"/>
       <c r="C32" s="15"/>
-      <c r="D32" s="49" t="s">
+      <c r="D32" s="53" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="50"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E32" s="54"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="1"/>
@@ -1699,7 +1691,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="2"/>
@@ -1711,7 +1703,7 @@
       <c r="I48" s="1"/>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="2"/>
@@ -1723,7 +1715,7 @@
       <c r="I49" s="1"/>
       <c r="J49" s="3"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="2"/>
@@ -1735,7 +1727,7 @@
       <c r="I50" s="1"/>
       <c r="J50" s="3"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="2"/>
@@ -1747,7 +1739,7 @@
       <c r="I51" s="1"/>
       <c r="J51" s="3"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1759,7 +1751,7 @@
       <c r="I52" s="1"/>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="2"/>
@@ -1771,7 +1763,7 @@
       <c r="I53" s="1"/>
       <c r="J53" s="3"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="2"/>
@@ -1816,12 +1808,11 @@
     <hyperlink ref="D29" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="D28" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="D31" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="C5" r:id="rId5" display="https://www.mouser.de/manufacturer/keystone/" xr:uid="{B1F4DA8D-BD2D-43B5-89B1-25ABF1C0529C}"/>
-    <hyperlink ref="J7" r:id="rId6" xr:uid="{E0F5E5CE-E58B-4232-8792-169F1500BA12}"/>
-    <hyperlink ref="J8" r:id="rId7" xr:uid="{85611FA3-DA6B-4401-BC4A-CB8B8F5F9061}"/>
+    <hyperlink ref="J8" r:id="rId5" xr:uid="{85611FA3-DA6B-4401-BC4A-CB8B8F5F9061}"/>
+    <hyperlink ref="C5" r:id="rId6" display="https://www.mouser.de/manufacturer/eagleplasticdevices/" xr:uid="{40DBAECB-FF27-46BD-9F79-41CFB06A3CDC}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId8"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId7"/>
   <headerFooter>
     <oddHeader>&amp;CParts list
 Practical Electronics</oddHeader>

</xml_diff>

<commit_message>
First draft of routing complete, parts list updated, 3d models added, button changed
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="13_ncr:1_{23A68183-9883-4898-B30F-B2C1DE7AC4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF5B5E48-CE05-4F58-8273-2AF4472BC6F5}"/>
+  <xr:revisionPtr revIDLastSave="133" documentId="13_ncr:1_{23A68183-9883-4898-B30F-B2C1DE7AC4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{038F8572-BD6D-4893-8699-53EA3B6121D6}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -222,21 +222,6 @@
     <t>Ceramic Capacitor 0.1uF</t>
   </si>
   <si>
-    <t>Push Button</t>
-  </si>
-  <si>
-    <t>https://www.mouser.de/ProductDetail/TE-Connectivity-PB/2-1977223-8?qs=WwRK9Mn48WC%252B3bZnlicO2g%3D%3D</t>
-  </si>
-  <si>
-    <t>506-2-1977223-8</t>
-  </si>
-  <si>
-    <t>2-1977223-8</t>
-  </si>
-  <si>
-    <t>TE Connectivity</t>
-  </si>
-  <si>
     <t>330 uH Inductor</t>
   </si>
   <si>
@@ -274,6 +259,21 @@
   </si>
   <si>
     <t>Eagle Plastic Devices</t>
+  </si>
+  <si>
+    <t>179-TS026660BK260LCR</t>
+  </si>
+  <si>
+    <t>TS02-66-60-BK-260-LCR-D</t>
+  </si>
+  <si>
+    <t>Push Button TS02-66-60-BK-260-LCR-D</t>
+  </si>
+  <si>
+    <t>Same Sky</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/Same-Sky/TS02-66-60-BK-260-LCR-D?qs=A6eO%252BMLsxmQnLv1ZYEDDrQ%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -677,6 +677,46 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -691,46 +731,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1059,38 +1059,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="43"/>
+      <c r="B1" s="48"/>
       <c r="C1" s="16" t="s">
         <v>34</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="43"/>
+      <c r="B2" s="48"/>
       <c r="C2" s="17">
         <v>45788</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="39" t="s">
+      <c r="H2" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
     </row>
     <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -1131,20 +1131,20 @@
       <c r="B5" s="18">
         <v>1</v>
       </c>
-      <c r="C5" s="55" t="s">
-        <v>79</v>
+      <c r="C5" s="38" t="s">
+        <v>74</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F5" s="18" t="s">
         <v>30</v>
       </c>
       <c r="G5" s="29" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="H5" s="23">
         <v>1.54</v>
@@ -1154,7 +1154,7 @@
         <v>1.54</v>
       </c>
       <c r="J5" s="22" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -1198,19 +1198,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="H7" s="25">
         <v>0.66200000000000003</v>
@@ -1220,7 +1220,7 @@
         <v>0.66200000000000003</v>
       </c>
       <c r="J7" s="26" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -1327,7 +1327,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>58</v>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="I11" s="24">
         <f t="shared" si="0"/>
-        <v>0.52</v>
+        <v>0.65</v>
       </c>
       <c r="J11" s="28" t="s">
         <v>57</v>
@@ -1363,29 +1363,29 @@
         <v>1</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="H12" s="25">
-        <v>0.16</v>
+        <v>8.5999999999999993E-2</v>
       </c>
       <c r="I12" s="24">
         <f t="shared" ref="I12:I13" si="1">B12*H12</f>
-        <v>0.16</v>
+        <v>8.5999999999999993E-2</v>
       </c>
       <c r="J12" s="26" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -1396,19 +1396,19 @@
         <v>1</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>30</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H13" s="25">
         <v>1.26</v>
@@ -1418,7 +1418,7 @@
         <v>1.26</v>
       </c>
       <c r="J13" s="26" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1562,13 +1562,13 @@
       <c r="J23" s="37"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G25" s="40" t="s">
+      <c r="G25" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="H25" s="40"/>
+      <c r="H25" s="54"/>
       <c r="I25" s="9">
         <f>SUM(I5:I23)</f>
-        <v>11.734999999999999</v>
+        <v>11.791</v>
       </c>
       <c r="J25" s="32"/>
     </row>
@@ -1580,104 +1580,104 @@
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
       <c r="E26" s="12"/>
-      <c r="G26" s="41" t="s">
+      <c r="G26" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="H26" s="41"/>
+      <c r="H26" s="55"/>
       <c r="I26" s="7">
         <f>I25*0.19</f>
-        <v>2.2296499999999999</v>
+        <v>2.2402899999999999</v>
       </c>
       <c r="J26" s="32"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="44" t="s">
+      <c r="A27" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="45"/>
+      <c r="B27" s="50"/>
       <c r="C27" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="45" t="s">
+      <c r="D27" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="48"/>
-      <c r="G27" s="41" t="s">
+      <c r="E27" s="51"/>
+      <c r="G27" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="H27" s="41"/>
+      <c r="H27" s="55"/>
       <c r="I27" s="8">
         <f>I25*1.19</f>
-        <v>13.964649999999999</v>
+        <v>14.03129</v>
       </c>
       <c r="J27" s="32"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="46" t="s">
+      <c r="A28" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="47"/>
+      <c r="B28" s="40"/>
       <c r="C28" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="51" t="s">
+      <c r="D28" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="E28" s="52"/>
+      <c r="E28" s="44"/>
       <c r="I28" s="31"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="46" t="s">
+      <c r="A29" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="47"/>
+      <c r="B29" s="40"/>
       <c r="C29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="51" t="s">
+      <c r="D29" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="52"/>
+      <c r="E29" s="44"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="46" t="s">
+      <c r="A30" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="47"/>
+      <c r="B30" s="40"/>
       <c r="C30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="51" t="s">
+      <c r="D30" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="E30" s="52"/>
+      <c r="E30" s="44"/>
       <c r="H30" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="49" t="s">
+      <c r="A31" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="50"/>
+      <c r="B31" s="42"/>
       <c r="C31" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="53" t="s">
+      <c r="D31" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="E31" s="54"/>
+      <c r="E31" s="46"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="49" t="s">
+      <c r="A32" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="50"/>
+      <c r="B32" s="42"/>
       <c r="C32" s="15"/>
-      <c r="D32" s="53" t="s">
+      <c r="D32" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="54"/>
+      <c r="E32" s="46"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
@@ -1777,6 +1777,16 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="D27:E27"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A32:B32"/>
@@ -1786,19 +1796,9 @@
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G27:H27"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F23 F16:F20 F5:F13" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$A$28:$A$32</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Updates to datasheet names
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -5,13 +5,13 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Projects\pe04\schematic-design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="133" documentId="13_ncr:1_{23A68183-9883-4898-B30F-B2C1DE7AC4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{038F8572-BD6D-4893-8699-53EA3B6121D6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B5337C-A70B-4C75-B714-785580CA96CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-60" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -678,45 +678,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -730,6 +691,45 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -747,10 +747,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1041,58 +1037,58 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J54"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="4.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="7.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="8" width="8.7109375" customWidth="1"/>
-    <col min="9" max="9" width="6.5703125" customWidth="1"/>
-    <col min="10" max="10" width="55.28515625" customWidth="1"/>
-    <col min="13" max="13" width="12.28515625" customWidth="1"/>
-    <col min="20" max="20" width="9.42578125" customWidth="1"/>
-    <col min="21" max="21" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" customWidth="1"/>
+    <col min="9" max="9" width="6.5546875" customWidth="1"/>
+    <col min="10" max="10" width="55.33203125" customWidth="1"/>
+    <col min="13" max="13" width="12.33203125" customWidth="1"/>
+    <col min="20" max="20" width="9.44140625" customWidth="1"/>
+    <col min="21" max="21" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="48"/>
+      <c r="B1" s="44"/>
       <c r="C1" s="16" t="s">
         <v>34</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="52" t="s">
+      <c r="H1" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="47" t="s">
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="48"/>
+      <c r="B2" s="44"/>
       <c r="C2" s="17">
         <v>45788</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="53" t="s">
+      <c r="H2" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-    </row>
-    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+    </row>
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -1124,7 +1120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>1</v>
       </c>
@@ -1157,7 +1153,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="6">
         <v>2</v>
       </c>
@@ -1190,7 +1186,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>3</v>
       </c>
@@ -1223,7 +1219,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="6">
         <v>4</v>
       </c>
@@ -1256,7 +1252,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>5</v>
       </c>
@@ -1289,7 +1285,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="6">
         <v>6</v>
       </c>
@@ -1322,7 +1318,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>7</v>
       </c>
@@ -1355,7 +1351,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="6">
         <v>8</v>
       </c>
@@ -1388,7 +1384,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>9</v>
       </c>
@@ -1421,7 +1417,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
         <v>10</v>
       </c>
@@ -1435,7 +1431,7 @@
       <c r="I14" s="34"/>
       <c r="J14" s="34"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>11</v>
       </c>
@@ -1449,7 +1445,7 @@
       <c r="I15" s="34"/>
       <c r="J15" s="34"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="6">
         <v>12</v>
       </c>
@@ -1463,7 +1459,7 @@
       <c r="I16" s="34"/>
       <c r="J16" s="34"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>13</v>
       </c>
@@ -1477,7 +1473,7 @@
       <c r="I17" s="34"/>
       <c r="J17" s="34"/>
     </row>
-    <row r="18" spans="1:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>14</v>
       </c>
@@ -1491,7 +1487,7 @@
       <c r="I18" s="34"/>
       <c r="J18" s="34"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>15</v>
       </c>
@@ -1505,7 +1501,7 @@
       <c r="I19" s="34"/>
       <c r="J19" s="34"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>16</v>
       </c>
@@ -1519,7 +1515,7 @@
       <c r="I20" s="34"/>
       <c r="J20" s="34"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>17</v>
       </c>
@@ -1533,7 +1529,7 @@
       <c r="I21" s="34"/>
       <c r="J21" s="34"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
         <v>18</v>
       </c>
@@ -1547,7 +1543,7 @@
       <c r="I22" s="34"/>
       <c r="J22" s="34"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>19</v>
       </c>
@@ -1561,18 +1557,18 @@
       <c r="I23" s="36"/>
       <c r="J23" s="37"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G25" s="54" t="s">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G25" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="H25" s="54"/>
+      <c r="H25" s="41"/>
       <c r="I25" s="9">
         <f>SUM(I5:I23)</f>
         <v>11.791</v>
       </c>
       <c r="J25" s="32"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>24</v>
       </c>
@@ -1580,106 +1576,106 @@
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
       <c r="E26" s="12"/>
-      <c r="G26" s="55" t="s">
+      <c r="G26" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="H26" s="55"/>
+      <c r="H26" s="42"/>
       <c r="I26" s="7">
         <f>I25*0.19</f>
         <v>2.2402899999999999</v>
       </c>
       <c r="J26" s="32"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="49" t="s">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="50"/>
+      <c r="B27" s="46"/>
       <c r="C27" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="51"/>
-      <c r="G27" s="55" t="s">
+      <c r="E27" s="49"/>
+      <c r="G27" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="H27" s="55"/>
+      <c r="H27" s="42"/>
       <c r="I27" s="8">
         <f>I25*1.19</f>
         <v>14.03129</v>
       </c>
       <c r="J27" s="32"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="39" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="40"/>
+      <c r="B28" s="48"/>
       <c r="C28" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="43" t="s">
+      <c r="D28" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="E28" s="44"/>
+      <c r="E28" s="53"/>
       <c r="I28" s="31"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="39" t="s">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="40"/>
+      <c r="B29" s="48"/>
       <c r="C29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="43" t="s">
+      <c r="D29" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="44"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="39" t="s">
+      <c r="E29" s="53"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="40"/>
+      <c r="B30" s="48"/>
       <c r="C30" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="43" t="s">
+      <c r="D30" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="E30" s="44"/>
+      <c r="E30" s="53"/>
       <c r="H30" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="41" t="s">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="42"/>
+      <c r="B31" s="51"/>
       <c r="C31" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="45" t="s">
+      <c r="D31" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="E31" s="46"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="41" t="s">
+      <c r="E31" s="55"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="42"/>
+      <c r="B32" s="51"/>
       <c r="C32" s="15"/>
-      <c r="D32" s="45" t="s">
+      <c r="D32" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="46"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E32" s="55"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="1"/>
@@ -1691,7 +1687,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="2"/>
@@ -1703,7 +1699,7 @@
       <c r="I48" s="1"/>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="2"/>
@@ -1715,7 +1711,7 @@
       <c r="I49" s="1"/>
       <c r="J49" s="3"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="2"/>
@@ -1727,7 +1723,7 @@
       <c r="I50" s="1"/>
       <c r="J50" s="3"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="2"/>
@@ -1739,7 +1735,7 @@
       <c r="I51" s="1"/>
       <c r="J51" s="3"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1751,7 +1747,7 @@
       <c r="I52" s="1"/>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="2"/>
@@ -1763,7 +1759,7 @@
       <c r="I53" s="1"/>
       <c r="J53" s="3"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="2"/>
@@ -1777,16 +1773,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="D27:E27"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A32:B32"/>
@@ -1796,6 +1782,16 @@
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G27:H27"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Final uploaded PCB design
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -5,13 +5,13 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Projects\pe04\schematic-design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070D2B56-7EFD-41E9-9606-CB84ABF9E623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{070D2B56-7EFD-41E9-9606-CB84ABF9E623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B34F81B8-0012-439C-948F-9DC267F397C4}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="76">
   <si>
     <t>Link</t>
   </si>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t>https://www.mouser.de/ProductDetail/Same-Sky/TS02-66-60-BK-260-LCR-D?qs=A6eO%252BMLsxmQnLv1ZYEDDrQ%3D%3D</t>
+  </si>
+  <si>
+    <t>19/11/2025</t>
   </si>
 </sst>
 </file>
@@ -705,6 +708,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1034,8 +1041,8 @@
         <v>21</v>
       </c>
       <c r="B2" s="45"/>
-      <c r="C2" s="17">
-        <v>45788</v>
+      <c r="C2" s="17" t="s">
+        <v>75</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>20</v>
@@ -1719,7 +1726,7 @@
     <mergeCell ref="D30:E30"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22 F5:F12 F15:F19" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$A$27:$A$31</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
3D Model updated, and code
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ad1c0a53281c2ab/Documents/University/Studies/Sem 5/Practical Electronics/pe04/schematic-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{070D2B56-7EFD-41E9-9606-CB84ABF9E623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B34F81B8-0012-439C-948F-9DC267F397C4}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{070D2B56-7EFD-41E9-9606-CB84ABF9E623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DC400CB-3153-4881-825A-6E92DDB5CB8E}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -639,45 +639,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -691,6 +652,45 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1020,38 +1020,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="45"/>
+      <c r="B1" s="41"/>
       <c r="C1" s="16" t="s">
         <v>34</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="49" t="s">
+      <c r="H1" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="45"/>
+      <c r="B2" s="41"/>
       <c r="C2" s="17" t="s">
         <v>75</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="50" t="s">
+      <c r="H2" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -1490,10 +1490,10 @@
       <c r="J22" s="34"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G24" s="51" t="s">
+      <c r="G24" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="H24" s="51"/>
+      <c r="H24" s="38"/>
       <c r="I24" s="9">
         <f>SUM(I5:I22)</f>
         <v>10.927000000000001</v>
@@ -1508,10 +1508,10 @@
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
       <c r="E25" s="12"/>
-      <c r="G25" s="52" t="s">
+      <c r="G25" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="H25" s="52"/>
+      <c r="H25" s="39"/>
       <c r="I25" s="7">
         <f>I24*0.19</f>
         <v>2.0761300000000005</v>
@@ -1519,21 +1519,21 @@
       <c r="J25" s="29"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="47"/>
+      <c r="B26" s="43"/>
       <c r="C26" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D26" s="47" t="s">
+      <c r="D26" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="E26" s="48"/>
-      <c r="G26" s="52" t="s">
+      <c r="E26" s="46"/>
+      <c r="G26" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="H26" s="52"/>
+      <c r="H26" s="39"/>
       <c r="I26" s="8">
         <f>I24*1.19</f>
         <v>13.003130000000001</v>
@@ -1541,71 +1541,71 @@
       <c r="J26" s="29"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="37"/>
+      <c r="B27" s="45"/>
       <c r="C27" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="40" t="s">
+      <c r="D27" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="41"/>
+      <c r="E27" s="50"/>
       <c r="I27" s="28"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="37"/>
+      <c r="B28" s="45"/>
       <c r="C28" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="40" t="s">
+      <c r="D28" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="41"/>
+      <c r="E28" s="50"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" s="36" t="s">
+      <c r="A29" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="37"/>
+      <c r="B29" s="45"/>
       <c r="C29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="40" t="s">
+      <c r="D29" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="E29" s="41"/>
+      <c r="E29" s="50"/>
       <c r="H29" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="38" t="s">
+      <c r="A30" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="39"/>
+      <c r="B30" s="48"/>
       <c r="C30" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="42" t="s">
+      <c r="D30" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="E30" s="43"/>
+      <c r="E30" s="52"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="38" t="s">
+      <c r="A31" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="39"/>
+      <c r="B31" s="48"/>
       <c r="C31" s="15"/>
-      <c r="D31" s="42" t="s">
+      <c r="D31" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="43"/>
+      <c r="E31" s="52"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
@@ -1705,16 +1705,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="D26:E26"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A31:B31"/>
@@ -1724,9 +1714,19 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G26:H26"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22 F5:F12 F15:F19" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$A$27:$A$31</formula1>
     </dataValidation>

</xml_diff>